<commit_message>
Protecting excel files with defused xml
</commit_message>
<xml_diff>
--- a/AutomatingMicrosoftExcel/StudentScores.xlsx
+++ b/AutomatingMicrosoftExcel/StudentScores.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t xml:space="preserve">Students</t>
   </si>
@@ -80,6 +80,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aq</t>
   </si>
 </sst>
 </file>
@@ -504,6 +507,9 @@
       <c r="D15" s="0" t="n">
         <v>25.5</v>
       </c>
+      <c r="F15" s="0" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>